<commit_message>
Modification du fichir Excel
retrait d'un back slash n
</commit_message>
<xml_diff>
--- a/data/velo.xlsx
+++ b/data/velo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Isen\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thier\Documents\Cour_isen_Année_3\Projet_fin_Année\Projet_Recherche_Operationnelle\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B470B69D-B2AB-46D5-A013-C41F9C8EAC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C97771-1D38-4FF7-93C5-B351DD35F7BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2570" yWindow="2860" windowWidth="14400" windowHeight="8170" xr2:uid="{AE980E81-492D-489C-A654-45A3CB44770F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE980E81-492D-489C-A654-45A3CB44770F}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -89,10 +89,6 @@
     <t>Arrache Manivelle</t>
   </si>
   <si>
-    <t>Bouchon valve 
-chromé bleu</t>
-  </si>
-  <si>
     <t>Rustines</t>
   </si>
   <si>
@@ -115,6 +111,9 @@
   </si>
   <si>
     <t>Veste de pluie</t>
+  </si>
+  <si>
+    <t>Bouchon valve chromé bleu</t>
   </si>
 </sst>
 </file>
@@ -515,14 +514,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CEF0C7E-6664-47A4-9C1A-134EDDAC2C49}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.08984375" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -531,7 +530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -542,7 +541,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -553,7 +552,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -564,7 +563,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -575,7 +574,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -586,7 +585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -597,7 +596,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -608,7 +607,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -619,7 +618,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -630,7 +629,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -641,9 +640,9 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="1">
         <v>0.4</v>
@@ -652,9 +651,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="1">
         <v>0.4</v>
@@ -663,7 +662,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -674,7 +673,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -685,7 +684,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -696,7 +695,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -707,9 +706,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" s="1">
         <v>0.3</v>
@@ -718,7 +717,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>16</v>
       </c>
@@ -729,9 +728,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B20" s="1">
         <v>0.01</v>
@@ -740,9 +739,9 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1">
         <v>0.05</v>
@@ -751,9 +750,9 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="1">
         <v>0.4</v>
@@ -762,9 +761,9 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="1">
         <v>0.6</v>
@@ -773,9 +772,9 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B24" s="1">
         <v>0.05</v>

</xml_diff>